<commit_message>
live update 13:18:14 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AD4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -714,6 +714,222 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>13:14:37</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0.6077</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>0.5739</v>
+      </c>
+      <c r="J3" t="n">
+        <v>8000</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5300</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="T3" s="2" t="n"/>
+      <c r="U3" s="2" t="n"/>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>0.008867220878601062</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>0.002265558242797866</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>13:16:10</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>0.656</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.598</v>
+      </c>
+      <c r="J4" t="n">
+        <v>12000</v>
+      </c>
+      <c r="K4" t="n">
+        <v>9100</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="V4" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W4" s="2" t="n">
+        <v>0.01199975252151489</v>
+      </c>
+      <c r="X4" s="2" t="n">
+        <v>0.003999505043029788</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 13:23:18 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -17,8 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -32,12 +34,24 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -52,10 +66,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD4"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -442,16 +461,16 @@
     <col width="6" customWidth="1" min="16" max="16"/>
     <col width="6" customWidth="1" min="17" max="17"/>
     <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="23" customWidth="1" min="23" max="23"/>
     <col width="23" customWidth="1" min="24" max="24"/>
-    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="25" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="8" customWidth="1" min="28" max="28"/>
+    <col width="30" customWidth="1" min="28" max="28"/>
     <col width="10" customWidth="1" min="29" max="29"/>
     <col width="9" customWidth="1" min="30" max="30"/>
   </cols>
@@ -925,6 +944,554 @@
         </is>
       </c>
       <c r="AD4" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>13:18:25</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>0.656</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>0.598</v>
+      </c>
+      <c r="J5" t="n">
+        <v>12000</v>
+      </c>
+      <c r="K5" t="n">
+        <v>9100</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>10</v>
+      </c>
+      <c r="O5" t="n">
+        <v>2</v>
+      </c>
+      <c r="P5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="V5" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W5" s="2" t="n">
+        <v>-0.008000247478485129</v>
+      </c>
+      <c r="X5" s="2" t="n">
+        <v>-0.03399950504302982</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>13:18:36</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0.7496</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0.6448</v>
+      </c>
+      <c r="J6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4200</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>15</v>
+      </c>
+      <c r="O6" t="n">
+        <v>4</v>
+      </c>
+      <c r="P6" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" t="n">
+        <v>3</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="V6" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W6" s="2" t="n">
+        <v>-0.01520942091941832</v>
+      </c>
+      <c r="X6" s="2" t="n">
+        <v>0.0595811581611633</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>13:21:01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0.8127</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>0.6763</v>
+      </c>
+      <c r="J7" t="n">
+        <v>6450</v>
+      </c>
+      <c r="K7" t="n">
+        <v>9300</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>19</v>
+      </c>
+      <c r="O7" t="n">
+        <v>6</v>
+      </c>
+      <c r="P7" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>0.5800000000000001</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="V7" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>0.04633368492126469</v>
+      </c>
+      <c r="X7" s="3" t="n">
+        <v>0.2126673698425293</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.570x175</t>
+        </is>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="4" t="inlineStr">
+        <is>
+          <t>BUY MAP1 ECSTATIC $100@0.570</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>13:23:06</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0.8127</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>0.6763</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6450</v>
+      </c>
+      <c r="K8" t="n">
+        <v>9300</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>19</v>
+      </c>
+      <c r="O8" t="n">
+        <v>6</v>
+      </c>
+      <c r="P8" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" t="n">
+        <v>4</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="U8" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="V8" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W8" s="2" t="n">
+        <v>-0.01366631507873536</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.570x175</t>
+        </is>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>13:23:17</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0.6983</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>0.6191</v>
+      </c>
+      <c r="J9" t="n">
+        <v>950</v>
+      </c>
+      <c r="K9" t="n">
+        <v>3400</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>19</v>
+      </c>
+      <c r="O9" t="n">
+        <v>8</v>
+      </c>
+      <c r="P9" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>2</v>
+      </c>
+      <c r="R9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="V9" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W9" s="2" t="n">
+        <v>-0.009149107933044437</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.570x175</t>
+        </is>
+      </c>
+      <c r="Z9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
         <is>
           <t>Nemesis</t>
         </is>
@@ -941,21 +1508,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
     <col width="5" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -1026,6 +1593,57 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>13:21:01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>175.4385964912281</v>
+      </c>
+      <c r="I2" s="6" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J2" s="6" t="n">
+        <v>0.8126673698425293</v>
+      </c>
+      <c r="K2" s="6" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="L2" s="6" t="n">
+        <v>0.2126673698425293</v>
+      </c>
+      <c r="M2" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 13:28:22 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -34,7 +34,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,12 @@
         <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -66,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -75,6 +81,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:AD15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -467,7 +475,7 @@
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="23" customWidth="1" min="23" max="23"/>
     <col width="23" customWidth="1" min="24" max="24"/>
-    <col width="25" customWidth="1" min="25" max="25"/>
+    <col width="29" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
     <col width="30" customWidth="1" min="28" max="28"/>
@@ -1492,6 +1500,666 @@
         </is>
       </c>
       <c r="AD9" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>13:24:20</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0.6983</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>0.6191</v>
+      </c>
+      <c r="J10" t="n">
+        <v>950</v>
+      </c>
+      <c r="K10" t="n">
+        <v>3400</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>19</v>
+      </c>
+      <c r="O10" t="n">
+        <v>8</v>
+      </c>
+      <c r="P10" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>2</v>
+      </c>
+      <c r="R10" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="T10" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="U10" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="V10" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W10" s="2" t="n">
+        <v>0.03085089206695554</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z10" t="n">
+        <v>26.32</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>31.58</v>
+      </c>
+      <c r="AB10" s="4" t="inlineStr">
+        <is>
+          <t>SELL MAP1 ECSTATIC P/L:$+26.32</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>13:24:31</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0.6351</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>0.5875</v>
+      </c>
+      <c r="J11" t="n">
+        <v>11650</v>
+      </c>
+      <c r="K11" t="n">
+        <v>9900</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>23</v>
+      </c>
+      <c r="O11" t="n">
+        <v>13</v>
+      </c>
+      <c r="P11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>3</v>
+      </c>
+      <c r="R11" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="U11" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="V11" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W11" s="2" t="n">
+        <v>0.06247282505035398</v>
+      </c>
+      <c r="X11" s="3" t="n">
+        <v>0.08494565010070801</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>MAP1:Team Nemesis@0.250x118</t>
+        </is>
+      </c>
+      <c r="Z11" t="n">
+        <v>26.32</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="4" t="inlineStr">
+        <is>
+          <t>BUY MAP1 Team Nemesis $30@0.250</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>13:26:15</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>7</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>6-2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>0.6351</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>0.5875</v>
+      </c>
+      <c r="J12" t="n">
+        <v>11650</v>
+      </c>
+      <c r="K12" t="n">
+        <v>9900</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>23</v>
+      </c>
+      <c r="O12" t="n">
+        <v>13</v>
+      </c>
+      <c r="P12" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>3</v>
+      </c>
+      <c r="R12" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="U12" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="V12" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W12" s="2" t="n">
+        <v>0.06247282505035398</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>MAP1:Team Nemesis@0.250x118</t>
+        </is>
+      </c>
+      <c r="Z12" t="n">
+        <v>26.32</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>-3.54</v>
+      </c>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>13:26:26</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>6-2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0.7924</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0.6662</v>
+      </c>
+      <c r="J13" t="n">
+        <v>2200</v>
+      </c>
+      <c r="K13" t="n">
+        <v>700</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>28</v>
+      </c>
+      <c r="O13" t="n">
+        <v>14</v>
+      </c>
+      <c r="P13" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>3</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="U13" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="V13" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W13" s="2" t="n">
+        <v>-0.01619103074073794</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>MAP1:Team Nemesis@0.250x118</t>
+        </is>
+      </c>
+      <c r="Z13" t="n">
+        <v>26.32</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>-3.54</v>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>13:27:29</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>7-2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0.7924</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>0.6662</v>
+      </c>
+      <c r="J14" t="n">
+        <v>2200</v>
+      </c>
+      <c r="K14" t="n">
+        <v>700</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>28</v>
+      </c>
+      <c r="O14" t="n">
+        <v>14</v>
+      </c>
+      <c r="P14" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>3</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="U14" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="V14" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W14" s="2" t="n">
+        <v>-0.01380896925926209</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z14" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="AB14" s="4" t="inlineStr">
+        <is>
+          <t>SELL MAP1 Team Nemesis P/L:$-2.36</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>13:27:40</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>9</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>7-2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0.8308</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>0.6854</v>
+      </c>
+      <c r="J15" t="n">
+        <v>4750</v>
+      </c>
+      <c r="K15" t="n">
+        <v>5200</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>33</v>
+      </c>
+      <c r="O15" t="n">
+        <v>14</v>
+      </c>
+      <c r="P15" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>3</v>
+      </c>
+      <c r="R15" t="n">
+        <v>2</v>
+      </c>
+      <c r="S15" s="2" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T15" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="U15" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="V15" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W15" s="2" t="n">
+        <v>0.005377527475357052</v>
+      </c>
+      <c r="X15" s="2" t="n">
+        <v>0.07075505495071413</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z15" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
         <is>
           <t>Nemesis</t>
         </is>
@@ -1508,7 +2176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1517,13 +2185,13 @@
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1642,6 +2310,159 @@
       </c>
       <c r="M2" s="7" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>13:24:20</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>175.4385964912281</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>0.6982982158660889</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>-0.05170178413391113</v>
+      </c>
+      <c r="M3" s="8" t="n">
+        <v>26.31578947368422</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>13:24:31</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Team Nemesis</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>118</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>0.364945650100708</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>0.465</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>0.08494565010070801</v>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>13:27:29</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Team Nemesis</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>118</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>0.2076179385185242</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>0.465</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>-0.05238206148147584</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>-2.359999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
live update 13:33:25 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD15"/>
+  <dimension ref="A1:AD19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2165,6 +2165,444 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>13:29:45</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>9</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>7-3</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0.8308</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>0.6854</v>
+      </c>
+      <c r="J16" t="n">
+        <v>4750</v>
+      </c>
+      <c r="K16" t="n">
+        <v>5200</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>33</v>
+      </c>
+      <c r="O16" t="n">
+        <v>14</v>
+      </c>
+      <c r="P16" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>3</v>
+      </c>
+      <c r="R16" t="n">
+        <v>2</v>
+      </c>
+      <c r="S16" s="2" t="n">
+        <v>0.695</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="U16" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="V16" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W16" s="2" t="n">
+        <v>-0.02537752747535707</v>
+      </c>
+      <c r="X16" s="2" t="n">
+        <v>0.01075505495071408</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="Z16" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>13:29:56</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>10</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>7-3</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>0.7125</v>
+      </c>
+      <c r="J17" t="n">
+        <v>7300</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>38</v>
+      </c>
+      <c r="O17" t="n">
+        <v>15</v>
+      </c>
+      <c r="P17" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>3</v>
+      </c>
+      <c r="R17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S17" s="2" t="n">
+        <v>0.695</v>
+      </c>
+      <c r="T17" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="U17" s="2" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="V17" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W17" s="2" t="n">
+        <v>-0.01751356482505792</v>
+      </c>
+      <c r="X17" s="3" t="n">
+        <v>0.09497287034988403</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z17" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB17" s="4" t="inlineStr">
+        <is>
+          <t>BUY MAP1 ECSTATIC $100@0.760</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13:30:59</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>10</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>8-3</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>0.7125</v>
+      </c>
+      <c r="J18" t="n">
+        <v>7300</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>38</v>
+      </c>
+      <c r="O18" t="n">
+        <v>15</v>
+      </c>
+      <c r="P18" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>3</v>
+      </c>
+      <c r="R18" t="n">
+        <v>3</v>
+      </c>
+      <c r="S18" s="2" t="n">
+        <v>0.675</v>
+      </c>
+      <c r="T18" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="U18" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="V18" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W18" s="2" t="n">
+        <v>0.002486435174941987</v>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z18" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>13:31:10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>11</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>8-3</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0.8061</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>0.6731</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1900</v>
+      </c>
+      <c r="K19" t="n">
+        <v>6500</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>39</v>
+      </c>
+      <c r="O19" t="n">
+        <v>20</v>
+      </c>
+      <c r="P19" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>4</v>
+      </c>
+      <c r="R19" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S19" s="2" t="n">
+        <v>0.675</v>
+      </c>
+      <c r="T19" s="2" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="U19" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="V19" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W19" s="2" t="n">
+        <v>-0.03307340025901798</v>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z19" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2176,7 +2614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2465,6 +2903,57 @@
         <v>-2.359999999999999</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>13:29:56</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>MAP1</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>131.578947368421</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>0.884972870349884</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>0.09497287034988403</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 13:38:31 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD19"/>
+  <dimension ref="A1:AD27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -475,7 +475,7 @@
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="23" customWidth="1" min="23" max="23"/>
     <col width="23" customWidth="1" min="24" max="24"/>
-    <col width="29" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="25" max="25"/>
     <col width="14" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
     <col width="30" customWidth="1" min="28" max="28"/>
@@ -2598,6 +2598,851 @@
         </is>
       </c>
       <c r="AD19" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>13:33:46</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>11</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>9-3</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>0.8061</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>0.6731</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1900</v>
+      </c>
+      <c r="K20" t="n">
+        <v>6500</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>39</v>
+      </c>
+      <c r="O20" t="n">
+        <v>20</v>
+      </c>
+      <c r="P20" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>4</v>
+      </c>
+      <c r="R20" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S20" s="2" t="n">
+        <v>0.665</v>
+      </c>
+      <c r="T20" s="2" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="U20" s="2" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="V20" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W20" s="2" t="n">
+        <v>-0.02692659974098208</v>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z20" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>-5.26</v>
+      </c>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>13:33:57</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>12</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>9-3</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>0.8722</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>0.7060999999999999</v>
+      </c>
+      <c r="J21" t="n">
+        <v>4450</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>44</v>
+      </c>
+      <c r="O21" t="n">
+        <v>24</v>
+      </c>
+      <c r="P21" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>4</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="T21" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="U21" s="2" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="V21" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W21" s="2" t="n">
+        <v>0.02607974052429199</v>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z21" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>-10.53</v>
+      </c>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>13:34:49</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>13</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>9-4</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>0.912</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>0.726</v>
+      </c>
+      <c r="J22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K22" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>49</v>
+      </c>
+      <c r="O22" t="n">
+        <v>28</v>
+      </c>
+      <c r="P22" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>4</v>
+      </c>
+      <c r="R22" t="n">
+        <v>2</v>
+      </c>
+      <c r="S22" s="2" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="T22" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="U22" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="V22" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W22" s="3" t="n">
+        <v>0.09600613951683049</v>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z22" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-21.05</v>
+      </c>
+      <c r="AB22" s="4" t="inlineStr">
+        <is>
+          <t>BUY WINNER ECSTATIC $58@0.600</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>13:35:31</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>13</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>9-5</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>0.912</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>0.726</v>
+      </c>
+      <c r="J23" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K23" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>49</v>
+      </c>
+      <c r="O23" t="n">
+        <v>28</v>
+      </c>
+      <c r="P23" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>4</v>
+      </c>
+      <c r="R23" t="n">
+        <v>2</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="T23" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="U23" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="V23" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z23" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>-23</v>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>13:35:42</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>14</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>9-5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>0.8495</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>0.6947</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="K24" t="n">
+        <v>6750</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>49</v>
+      </c>
+      <c r="O24" t="n">
+        <v>33</v>
+      </c>
+      <c r="P24" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>5</v>
+      </c>
+      <c r="R24" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S24" s="2" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="T24" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="U24" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="V24" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z24" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>-25.63</v>
+      </c>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>13:36:24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>14</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>9-6</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>0.8495</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>0.6947</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="K25" t="n">
+        <v>6750</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>49</v>
+      </c>
+      <c r="O25" t="n">
+        <v>33</v>
+      </c>
+      <c r="P25" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>5</v>
+      </c>
+      <c r="R25" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>0.585</v>
+      </c>
+      <c r="T25" s="2" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="U25" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="V25" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z25" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>-29.58</v>
+      </c>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:36:35</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>15</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>9-6</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>0.7887999999999999</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>0.6644</v>
+      </c>
+      <c r="J26" t="n">
+        <v>800</v>
+      </c>
+      <c r="K26" t="n">
+        <v>9500</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>50</v>
+      </c>
+      <c r="O26" t="n">
+        <v>38</v>
+      </c>
+      <c r="P26" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>6</v>
+      </c>
+      <c r="R26" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="T26" s="2" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="U26" s="2" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="V26" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z26" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>-30.55</v>
+      </c>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>13:38:30</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>16</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>9-7</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>0.7226</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>0.6313</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3100</v>
+      </c>
+      <c r="K27" t="n">
+        <v>12250</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>51</v>
+      </c>
+      <c r="O27" t="n">
+        <v>43</v>
+      </c>
+      <c r="P27" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>7</v>
+      </c>
+      <c r="R27" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T27" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="U27" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="V27" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z27" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>-58.07</v>
+      </c>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
         <is>
           <t>Nemesis</t>
         </is>
@@ -2614,7 +3459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2954,6 +3799,57 @@
         <v>0</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>13:34:49</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>13</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>WINNER</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>97.30500000000001</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>0.7260061395168305</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>0.09600613951683049</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 13:43:35 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD27"/>
+  <dimension ref="A1:AD31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3448,6 +3448,422 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:40:15</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>16</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>9-8</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>0.7226</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>0.6313</v>
+      </c>
+      <c r="J28" t="n">
+        <v>3100</v>
+      </c>
+      <c r="K28" t="n">
+        <v>12250</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>51</v>
+      </c>
+      <c r="O28" t="n">
+        <v>43</v>
+      </c>
+      <c r="P28" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>7</v>
+      </c>
+      <c r="R28" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S28" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T28" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="U28" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="V28" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z28" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>-59.39</v>
+      </c>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:40:26</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>17</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>9-8</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>0.6005</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>0.5703</v>
+      </c>
+      <c r="J29" t="n">
+        <v>7900</v>
+      </c>
+      <c r="K29" t="n">
+        <v>3000</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>52</v>
+      </c>
+      <c r="O29" t="n">
+        <v>48</v>
+      </c>
+      <c r="P29" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>8</v>
+      </c>
+      <c r="R29" t="n">
+        <v>-4</v>
+      </c>
+      <c r="S29" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="T29" s="2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="U29" s="2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="V29" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z29" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>-59.39</v>
+      </c>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:43:02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>17</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>9-9</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>0.6005</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>0.5703</v>
+      </c>
+      <c r="J30" t="n">
+        <v>7900</v>
+      </c>
+      <c r="K30" t="n">
+        <v>3000</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
+        <v>52</v>
+      </c>
+      <c r="O30" t="n">
+        <v>48</v>
+      </c>
+      <c r="P30" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>8</v>
+      </c>
+      <c r="R30" t="n">
+        <v>-4</v>
+      </c>
+      <c r="S30" s="2" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="T30" s="2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="U30" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="V30" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z30" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>-96.12</v>
+      </c>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>13:43:13</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>18</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>9-9</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>0.5152</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>0.5276</v>
+      </c>
+      <c r="J31" t="n">
+        <v>900</v>
+      </c>
+      <c r="K31" t="n">
+        <v>5550</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>52</v>
+      </c>
+      <c r="O31" t="n">
+        <v>53</v>
+      </c>
+      <c r="P31" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>9</v>
+      </c>
+      <c r="R31" t="n">
+        <v>-5</v>
+      </c>
+      <c r="S31" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="T31" s="2" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="U31" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="V31" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z31" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>-95.43000000000001</v>
+      </c>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 13:48:38 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD31"/>
+  <dimension ref="A1:AD34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3864,6 +3864,318 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>13:45:19</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>19</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>9-10</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>0.3779</v>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="J32" t="n">
+        <v>5700</v>
+      </c>
+      <c r="K32" t="n">
+        <v>7900</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>53</v>
+      </c>
+      <c r="O32" t="n">
+        <v>58</v>
+      </c>
+      <c r="P32" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>10</v>
+      </c>
+      <c r="R32" t="n">
+        <v>-6</v>
+      </c>
+      <c r="S32" s="2" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="T32" s="2" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="U32" s="2" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="V32" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z32" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>-103.96</v>
+      </c>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>13:47:13</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>19</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>9-11</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n">
+        <v>0.3779</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="J33" t="n">
+        <v>5700</v>
+      </c>
+      <c r="K33" t="n">
+        <v>7900</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>53</v>
+      </c>
+      <c r="O33" t="n">
+        <v>58</v>
+      </c>
+      <c r="P33" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>10</v>
+      </c>
+      <c r="R33" t="n">
+        <v>-6</v>
+      </c>
+      <c r="S33" s="2" t="n">
+        <v>0.335</v>
+      </c>
+      <c r="T33" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="U33" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="V33" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z33" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>-121.01</v>
+      </c>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>13:47:24</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>20</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>9-11</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>0.2664</v>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>0.4032</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>10450</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>55</v>
+      </c>
+      <c r="O34" t="n">
+        <v>63</v>
+      </c>
+      <c r="P34" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>11</v>
+      </c>
+      <c r="R34" t="n">
+        <v>-7</v>
+      </c>
+      <c r="S34" s="2" t="n">
+        <v>0.335</v>
+      </c>
+      <c r="T34" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="U34" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="V34" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:ECSTATIC@0.600x97</t>
+        </is>
+      </c>
+      <c r="Z34" t="n">
+        <v>23.96</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>-122.32</v>
+      </c>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 13:53:43 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD34"/>
+  <dimension ref="A1:AD37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4176,6 +4176,332 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>13:49:30</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>20</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="n">
+        <v>0.2664</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>0.4032</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>10450</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
+        <v>55</v>
+      </c>
+      <c r="O35" t="n">
+        <v>63</v>
+      </c>
+      <c r="P35" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>11</v>
+      </c>
+      <c r="R35" t="n">
+        <v>-7</v>
+      </c>
+      <c r="S35" s="2" t="n">
+        <v>0.305</v>
+      </c>
+      <c r="T35" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="U35" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V35" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z35" t="n">
+        <v>-8.15</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>-29.19</v>
+      </c>
+      <c r="AB35" s="4" t="inlineStr">
+        <is>
+          <t>FORCE-EXIT WINNER ECSTATIC P/L:$-32.11</t>
+        </is>
+      </c>
+      <c r="AC35" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>13:49:41</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>21</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>0.1226</v>
+      </c>
+      <c r="I36" s="2" t="n">
+        <v>0.3313</v>
+      </c>
+      <c r="J36" t="n">
+        <v>9100</v>
+      </c>
+      <c r="K36" t="n">
+        <v>2450</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N36" t="n">
+        <v>57</v>
+      </c>
+      <c r="O36" t="n">
+        <v>68</v>
+      </c>
+      <c r="P36" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>12</v>
+      </c>
+      <c r="R36" t="n">
+        <v>-8</v>
+      </c>
+      <c r="S36" s="2" t="n">
+        <v>0.305</v>
+      </c>
+      <c r="T36" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="U36" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V36" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W36" s="2" t="n">
+        <v>-0.008688457012176493</v>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z36" t="n">
+        <v>-8.15</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>13:51:15</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>22</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>9-13</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>0.054</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="J37" t="n">
+        <v>3000</v>
+      </c>
+      <c r="K37" t="n">
+        <v>4800</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N37" t="n">
+        <v>60</v>
+      </c>
+      <c r="O37" t="n">
+        <v>73</v>
+      </c>
+      <c r="P37" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>13</v>
+      </c>
+      <c r="R37" t="n">
+        <v>-9</v>
+      </c>
+      <c r="S37" s="2" t="n">
+        <v>0.315</v>
+      </c>
+      <c r="T37" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="U37" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="V37" t="n">
+        <v>5170.6616</v>
+      </c>
+      <c r="W37" s="3" t="n">
+        <v>0.2529854930192232</v>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:Team Nemesis@0.690x130; O/U:Under@0.520x156</t>
+        </is>
+      </c>
+      <c r="Z37" t="n">
+        <v>-8.15</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB37" s="4" t="inlineStr">
+        <is>
+          <t>BUY WINNER Team Nemesis $90@0.690  BUY O/U Under $81@0.520</t>
+        </is>
+      </c>
+      <c r="AC37" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4187,7 +4513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4195,7 +4521,7 @@
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
@@ -4578,6 +4904,159 @@
         <v>0</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>13:49:30</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>WINNER</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>FORCE-EXIT</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>97.30500000000001</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>0.4031879496574402</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>0.1031879496574402</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>-32.11065</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>13:51:15</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>22</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>WINNER</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Team Nemesis</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>130.4347826086957</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>0.9729854930192232</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>0.465</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0.2529854930192232</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>13:51:15</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>22</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>mirage</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>O/U</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Under</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>155.7692307692308</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>0.9459709860384464</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>0.3959709860384464</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 14:14:00 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,13 +448,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD37"/>
+  <dimension ref="A1:AD42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
@@ -469,10 +469,10 @@
     <col width="6" customWidth="1" min="16" max="16"/>
     <col width="6" customWidth="1" min="17" max="17"/>
     <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
     <col width="23" customWidth="1" min="23" max="23"/>
     <col width="23" customWidth="1" min="24" max="24"/>
     <col width="30" customWidth="1" min="25" max="25"/>
@@ -4502,6 +4502,545 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>14:10:05</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>0.5585</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>0.2792</v>
+      </c>
+      <c r="J38" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K38" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" s="2" t="n">
+        <v>0.315</v>
+      </c>
+      <c r="T38" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="U38" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="V38" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="X38" s="2" t="n">
+        <v>-0.04152510166168208</v>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:Team Nemesis@0.690x130; O/U:Under@0.520x156</t>
+        </is>
+      </c>
+      <c r="Z38" t="n">
+        <v>-8.15</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>-29.34</v>
+      </c>
+      <c r="AB38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>14:11:50</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>0.5585</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>0.2792</v>
+      </c>
+      <c r="J39" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K39" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" s="2" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="T39" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="U39" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="V39" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="X39" s="2" t="n">
+        <v>-0.04152510166168208</v>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; WINNER:Team Nemesis@0.690x130; O/U:Under@0.520x156</t>
+        </is>
+      </c>
+      <c r="Z39" t="n">
+        <v>-8.15</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>-5.43</v>
+      </c>
+      <c r="AB39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>14:12:01</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>0.6813</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>0.3407</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
+        <v>11600</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>5</v>
+      </c>
+      <c r="O40" t="n">
+        <v>2</v>
+      </c>
+      <c r="P40" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" t="n">
+        <v>1</v>
+      </c>
+      <c r="S40" s="2" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="T40" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="U40" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="V40" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="X40" s="3" t="n">
+        <v>0.2113291907310486</v>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.440x186</t>
+        </is>
+      </c>
+      <c r="Z40" t="n">
+        <v>-15.94</v>
+      </c>
+      <c r="AA40" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AB40" s="4" t="inlineStr">
+        <is>
+          <t>SELL WINNER Team Nemesis P/L:$+0.00  BUY MAP2 ECSTATIC $82@0.440  SELL O/U Under P/L:$-7.79</t>
+        </is>
+      </c>
+      <c r="AC40" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>14:13:47</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>0.6813</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>0.3407</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
+        <v>11600</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
+        <v>5</v>
+      </c>
+      <c r="O41" t="n">
+        <v>2</v>
+      </c>
+      <c r="P41" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" t="n">
+        <v>1</v>
+      </c>
+      <c r="S41" s="2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="T41" s="2" t="n"/>
+      <c r="U41" s="2" t="n"/>
+      <c r="V41" t="n">
+        <v>0</v>
+      </c>
+      <c r="W41" s="2" t="n">
+        <v>-0.01933540463447572</v>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.440x186; O/U:Over@0.410x58</t>
+        </is>
+      </c>
+      <c r="Z41" t="n">
+        <v>-15.94</v>
+      </c>
+      <c r="AA41" t="n">
+        <v>-24.12</v>
+      </c>
+      <c r="AB41" s="4" t="inlineStr">
+        <is>
+          <t>BUY O/U Over $24@0.410</t>
+        </is>
+      </c>
+      <c r="AC41" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>14:13:58</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>0.5024999999999999</v>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>0.2513</v>
+      </c>
+      <c r="J42" t="n">
+        <v>1900</v>
+      </c>
+      <c r="K42" t="n">
+        <v>4800</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
+        <v>8</v>
+      </c>
+      <c r="O42" t="n">
+        <v>7</v>
+      </c>
+      <c r="P42" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>1</v>
+      </c>
+      <c r="R42" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S42" s="2" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="T42" s="2" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="U42" s="2" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="V42" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W42" s="2" t="n">
+        <v>0.001256376504898071</v>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.440x186; O/U:Over@0.410x58</t>
+        </is>
+      </c>
+      <c r="Z42" t="n">
+        <v>-15.94</v>
+      </c>
+      <c r="AA42" t="n">
+        <v>-31.62</v>
+      </c>
+      <c r="AB42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4513,13 +5052,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
@@ -4527,7 +5066,7 @@
     <col width="7" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -5057,6 +5596,210 @@
         <v>0</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>14:12:01</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>WINNER</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Team Nemesis</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>130.4347826086957</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>0.6593354046344757</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>0.6699999999999999</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>-0.06066459536552427</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>14:12:01</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>MAP2</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>185.5407272727273</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>0.6813291907310486</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>0.2113291907310486</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>14:12:01</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>O/U</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Under</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>155.7692307692308</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>0.3186708092689514</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>-0.1813291907310486</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>-7.788461538461545</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>14:13:47</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>O/U</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>57.66458656390245</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>0.6813291907310486</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>0.2413291907310486</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 14:19:07 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD42"/>
+  <dimension ref="A1:AD46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5041,6 +5041,438 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>14:14:42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>0.212</v>
+      </c>
+      <c r="J43" t="n">
+        <v>1700</v>
+      </c>
+      <c r="K43" t="n">
+        <v>8450</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>9</v>
+      </c>
+      <c r="O43" t="n">
+        <v>12</v>
+      </c>
+      <c r="P43" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>2</v>
+      </c>
+      <c r="R43" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S43" s="2" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="T43" s="2" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="U43" s="2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="V43" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W43" s="2" t="n">
+        <v>-0.0319834274053574</v>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.440x186; O/U:Over@0.410x58</t>
+        </is>
+      </c>
+      <c r="Z43" t="n">
+        <v>-15.94</v>
+      </c>
+      <c r="AA43" t="n">
+        <v>-26.75</v>
+      </c>
+      <c r="AB43" t="inlineStr"/>
+      <c r="AC43" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>14:15:56</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>5</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>0.4021</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>0.2011</v>
+      </c>
+      <c r="J44" t="n">
+        <v>3700</v>
+      </c>
+      <c r="K44" t="n">
+        <v>11200</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>9</v>
+      </c>
+      <c r="O44" t="n">
+        <v>17</v>
+      </c>
+      <c r="P44" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>3</v>
+      </c>
+      <c r="R44" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S44" s="2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="T44" s="2" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="U44" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="V44" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W44" s="2" t="n">
+        <v>0.01894939064979553</v>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.440x186; O/U:Over@0.410x58</t>
+        </is>
+      </c>
+      <c r="Z44" t="n">
+        <v>-15.94</v>
+      </c>
+      <c r="AA44" t="n">
+        <v>-4.16</v>
+      </c>
+      <c r="AB44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>14:17:41</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>5</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>0.4021</v>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>0.2011</v>
+      </c>
+      <c r="J45" t="n">
+        <v>3700</v>
+      </c>
+      <c r="K45" t="n">
+        <v>11200</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>9</v>
+      </c>
+      <c r="O45" t="n">
+        <v>17</v>
+      </c>
+      <c r="P45" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>3</v>
+      </c>
+      <c r="R45" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S45" s="2" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="T45" s="2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="U45" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="V45" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W45" s="2" t="n">
+        <v>-0.03105060935020451</v>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.440x186; O/U:Over@0.410x58</t>
+        </is>
+      </c>
+      <c r="Z45" t="n">
+        <v>-15.94</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>-21.31</v>
+      </c>
+      <c r="AB45" t="inlineStr"/>
+      <c r="AC45" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>14:17:53</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>6</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>0.3034</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>0.1517</v>
+      </c>
+      <c r="J46" t="n">
+        <v>8800</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1950</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>11</v>
+      </c>
+      <c r="O46" t="n">
+        <v>22</v>
+      </c>
+      <c r="P46" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>3</v>
+      </c>
+      <c r="R46" t="n">
+        <v>-4</v>
+      </c>
+      <c r="S46" s="2" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="T46" s="2" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="U46" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="V46" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W46" s="2" t="n">
+        <v>0.01828451275825496</v>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; O/U:Over@0.410x58</t>
+        </is>
+      </c>
+      <c r="Z46" t="n">
+        <v>-38.21</v>
+      </c>
+      <c r="AA46" t="n">
+        <v>-21.89</v>
+      </c>
+      <c r="AB46" s="4" t="inlineStr">
+        <is>
+          <t>SELL MAP2 ECSTATIC P/L:$-22.26</t>
+        </is>
+      </c>
+      <c r="AC46" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5052,7 +5484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5800,6 +6232,57 @@
         <v>0</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>14:17:53</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>6</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>MAP2</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>185.5407272727273</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>0.30343097448349</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>-0.04656902551650999</v>
+      </c>
+      <c r="M15" s="9" t="n">
+        <v>-22.26488727272728</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 14:24:15 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD46"/>
+  <dimension ref="A1:AD50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5473,6 +5473,444 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>14:20:00</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>6</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2-5</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>0.3034</v>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>0.1517</v>
+      </c>
+      <c r="J47" t="n">
+        <v>8800</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1950</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>11</v>
+      </c>
+      <c r="O47" t="n">
+        <v>22</v>
+      </c>
+      <c r="P47" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>3</v>
+      </c>
+      <c r="R47" t="n">
+        <v>-4</v>
+      </c>
+      <c r="S47" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="T47" s="2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="U47" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="V47" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W47" s="2" t="n">
+        <v>-0.02171548724174496</v>
+      </c>
+      <c r="X47" s="2" t="n">
+        <v>-0.01656902551650999</v>
+      </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; O/U:Over@0.410x58</t>
+        </is>
+      </c>
+      <c r="Z47" t="n">
+        <v>-38.21</v>
+      </c>
+      <c r="AA47" t="n">
+        <v>-9.800000000000001</v>
+      </c>
+      <c r="AB47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>14:20:11</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>7</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2-5</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>0.4591</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>0.2296</v>
+      </c>
+      <c r="J48" t="n">
+        <v>3200</v>
+      </c>
+      <c r="K48" t="n">
+        <v>9250</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>14</v>
+      </c>
+      <c r="O48" t="n">
+        <v>23</v>
+      </c>
+      <c r="P48" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>3</v>
+      </c>
+      <c r="R48" t="n">
+        <v>1</v>
+      </c>
+      <c r="S48" s="2" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="T48" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="U48" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="V48" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W48" s="2" t="n">
+        <v>0.02957275807857512</v>
+      </c>
+      <c r="X48" s="3" t="n">
+        <v>0.1391455161571503</v>
+      </c>
+      <c r="Y48" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; O/U:Over@0.410x58; MAP2:ECSTATIC@0.290x155</t>
+        </is>
+      </c>
+      <c r="Z48" t="n">
+        <v>-38.21</v>
+      </c>
+      <c r="AA48" t="n">
+        <v>-8.65</v>
+      </c>
+      <c r="AB48" s="4" t="inlineStr">
+        <is>
+          <t>BUY MAP2 ECSTATIC $45@0.290</t>
+        </is>
+      </c>
+      <c r="AC48" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>14:22:17</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>7</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="n">
+        <v>0.4591</v>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>0.2296</v>
+      </c>
+      <c r="J49" t="n">
+        <v>3200</v>
+      </c>
+      <c r="K49" t="n">
+        <v>9250</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>14</v>
+      </c>
+      <c r="O49" t="n">
+        <v>23</v>
+      </c>
+      <c r="P49" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>3</v>
+      </c>
+      <c r="R49" t="n">
+        <v>1</v>
+      </c>
+      <c r="S49" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="T49" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="U49" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V49" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W49" s="2" t="n">
+        <v>0.02957275807857512</v>
+      </c>
+      <c r="Y49" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; O/U:Over@0.410x58; MAP2:ECSTATIC@0.290x155</t>
+        </is>
+      </c>
+      <c r="Z49" t="n">
+        <v>-38.21</v>
+      </c>
+      <c r="AA49" t="n">
+        <v>-17.14</v>
+      </c>
+      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>14:22:29</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>8</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2-6</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>0.3405</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>0.1702</v>
+      </c>
+      <c r="J50" t="n">
+        <v>8300</v>
+      </c>
+      <c r="K50" t="n">
+        <v>11300</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>16</v>
+      </c>
+      <c r="O50" t="n">
+        <v>27</v>
+      </c>
+      <c r="P50" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>4</v>
+      </c>
+      <c r="R50" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S50" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="T50" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="U50" s="2" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="V50" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W50" s="2" t="n">
+        <v>-0.01975311577320099</v>
+      </c>
+      <c r="Y50" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; O/U:Over@0.410x58; MAP2:ECSTATIC@0.290x155</t>
+        </is>
+      </c>
+      <c r="Z50" t="n">
+        <v>-38.21</v>
+      </c>
+      <c r="AA50" t="n">
+        <v>-23.51</v>
+      </c>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5484,7 +5922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6283,6 +6721,57 @@
         <v>-22.26488727272728</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>14:20:11</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>7</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>MAP2</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>154.6015541312766</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>0.4591455161571503</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>0.1391455161571503</v>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 14:29:22 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD50"/>
+  <dimension ref="A1:AD54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5911,6 +5911,452 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>14:24:46</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>8</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2-7</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="n">
+        <v>0.3405</v>
+      </c>
+      <c r="I51" s="2" t="n">
+        <v>0.1702</v>
+      </c>
+      <c r="J51" t="n">
+        <v>8300</v>
+      </c>
+      <c r="K51" t="n">
+        <v>11300</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>16</v>
+      </c>
+      <c r="O51" t="n">
+        <v>27</v>
+      </c>
+      <c r="P51" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>4</v>
+      </c>
+      <c r="R51" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S51" s="2" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="T51" s="2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="U51" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="V51" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W51" s="2" t="n">
+        <v>-0.03024688422679897</v>
+      </c>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; O/U:Over@0.410x58; MAP2:ECSTATIC@0.290x155</t>
+        </is>
+      </c>
+      <c r="Z51" t="n">
+        <v>-38.21</v>
+      </c>
+      <c r="AA51" t="n">
+        <v>-13.08</v>
+      </c>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>14:24:58</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>9</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2-7</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>0.2247</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>0.1123</v>
+      </c>
+      <c r="J52" t="n">
+        <v>1900</v>
+      </c>
+      <c r="K52" t="n">
+        <v>1850</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
+        <v>18</v>
+      </c>
+      <c r="O52" t="n">
+        <v>32</v>
+      </c>
+      <c r="P52" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>5</v>
+      </c>
+      <c r="R52" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S52" s="2" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="T52" s="2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="U52" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="V52" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W52" s="2" t="n">
+        <v>0.02767159730196003</v>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; O/U:Over@0.410x58</t>
+        </is>
+      </c>
+      <c r="Z52" t="n">
+        <v>-44.39</v>
+      </c>
+      <c r="AA52" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="AB52" s="4" t="inlineStr">
+        <is>
+          <t>SELL MAP2 ECSTATIC P/L:$-6.18</t>
+        </is>
+      </c>
+      <c r="AC52" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>14:27:25</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>10</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>3-7</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>0.1586</v>
+      </c>
+      <c r="I53" s="2" t="n">
+        <v>0.0793</v>
+      </c>
+      <c r="J53" t="n">
+        <v>6700</v>
+      </c>
+      <c r="K53" t="n">
+        <v>4200</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>19</v>
+      </c>
+      <c r="O53" t="n">
+        <v>37</v>
+      </c>
+      <c r="P53" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>6</v>
+      </c>
+      <c r="R53" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S53" s="2" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="T53" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="U53" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="V53" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W53" s="2" t="n">
+        <v>-0.009309985041618368</v>
+      </c>
+      <c r="X53" s="2" t="n">
+        <v>0.02138002991676327</v>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z53" t="n">
+        <v>-56.5</v>
+      </c>
+      <c r="AA53" t="n">
+        <v>-10.38</v>
+      </c>
+      <c r="AB53" s="4" t="inlineStr">
+        <is>
+          <t>SELL O/U Over P/L:$-12.11</t>
+        </is>
+      </c>
+      <c r="AC53" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>14:29:10</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>11</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>3-8</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>0.2641</v>
+      </c>
+      <c r="I54" s="2" t="n">
+        <v>0.132</v>
+      </c>
+      <c r="J54" t="n">
+        <v>1400</v>
+      </c>
+      <c r="K54" t="n">
+        <v>11800</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N54" t="n">
+        <v>23</v>
+      </c>
+      <c r="O54" t="n">
+        <v>39</v>
+      </c>
+      <c r="P54" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>7</v>
+      </c>
+      <c r="R54" t="n">
+        <v>1</v>
+      </c>
+      <c r="S54" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="T54" s="2" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="U54" s="2" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="V54" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W54" s="2" t="n">
+        <v>-0.007962211370468139</v>
+      </c>
+      <c r="X54" s="3" t="n">
+        <v>0.08407557725906373</v>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.150x154</t>
+        </is>
+      </c>
+      <c r="Z54" t="n">
+        <v>-56.5</v>
+      </c>
+      <c r="AA54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB54" s="4" t="inlineStr">
+        <is>
+          <t>BUY MAP2 ECSTATIC $23@0.150</t>
+        </is>
+      </c>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5922,7 +6368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5937,7 +6383,7 @@
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6769,6 +7215,159 @@
         <v>0.1391455161571503</v>
       </c>
       <c r="M16" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>14:24:58</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>9</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>MAP2</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>154.6015541312766</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>0.22465680539608</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>-0.05534319460392001</v>
+      </c>
+      <c r="M17" s="9" t="n">
+        <v>-6.18406216525106</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>14:27:25</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>O/U</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>57.66458656390245</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>0.1586199700832367</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>-0.07138002991676332</v>
+      </c>
+      <c r="M18" s="9" t="n">
+        <v>-12.10956317841951</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>14:29:10</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>11</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>MAP2</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>153.78</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>0.2640755772590637</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>0.08407557725906373</v>
+      </c>
+      <c r="M19" s="7" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
live update 14:34:31 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD54"/>
+  <dimension ref="A1:AD59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6357,6 +6357,543 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>14:30:56</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>11</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>3-9</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>0.2641</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>0.132</v>
+      </c>
+      <c r="J55" t="n">
+        <v>1400</v>
+      </c>
+      <c r="K55" t="n">
+        <v>11800</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N55" t="n">
+        <v>23</v>
+      </c>
+      <c r="O55" t="n">
+        <v>39</v>
+      </c>
+      <c r="P55" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>7</v>
+      </c>
+      <c r="R55" t="n">
+        <v>1</v>
+      </c>
+      <c r="S55" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="T55" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="U55" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="V55" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W55" s="2" t="n">
+        <v>0.05203778862953186</v>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.150x154; O/U:Over@0.120x129</t>
+        </is>
+      </c>
+      <c r="Z55" t="n">
+        <v>-56.5</v>
+      </c>
+      <c r="AA55" t="n">
+        <v>-16.92</v>
+      </c>
+      <c r="AB55" s="4" t="inlineStr">
+        <is>
+          <t>BUY O/U Over $15@0.120</t>
+        </is>
+      </c>
+      <c r="AC55" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD55" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>14:31:08</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>12</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>3-9</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>0.1617</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>0.0809</v>
+      </c>
+      <c r="J56" t="n">
+        <v>5900</v>
+      </c>
+      <c r="K56" t="n">
+        <v>2550</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N56" t="n">
+        <v>23</v>
+      </c>
+      <c r="O56" t="n">
+        <v>44</v>
+      </c>
+      <c r="P56" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>8</v>
+      </c>
+      <c r="R56" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S56" s="2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="T56" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="U56" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="V56" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W56" s="2" t="n">
+        <v>0.0008522924780845625</v>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.150x154; O/U:Over@0.120x129</t>
+        </is>
+      </c>
+      <c r="Z56" t="n">
+        <v>-56.5</v>
+      </c>
+      <c r="AA56" t="n">
+        <v>-31.36</v>
+      </c>
+      <c r="AB56" t="inlineStr"/>
+      <c r="AC56" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD56" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>14:32:22</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>12</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>3-10</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="n">
+        <v>0.1617</v>
+      </c>
+      <c r="I57" s="2" t="n">
+        <v>0.0809</v>
+      </c>
+      <c r="J57" t="n">
+        <v>5900</v>
+      </c>
+      <c r="K57" t="n">
+        <v>2550</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
+        <v>23</v>
+      </c>
+      <c r="O57" t="n">
+        <v>44</v>
+      </c>
+      <c r="P57" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>8</v>
+      </c>
+      <c r="R57" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S57" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="T57" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="U57" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="V57" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W57" s="2" t="n">
+        <v>0.02085229247808457</v>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.150x154; O/U:Over@0.120x129</t>
+        </is>
+      </c>
+      <c r="Z57" t="n">
+        <v>-56.5</v>
+      </c>
+      <c r="AA57" t="n">
+        <v>-29.82</v>
+      </c>
+      <c r="AB57" t="inlineStr"/>
+      <c r="AC57" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD57" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>14:32:34</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>13</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>3-10</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>0.0873</v>
+      </c>
+      <c r="I58" s="2" t="n">
+        <v>0.0436</v>
+      </c>
+      <c r="J58" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K58" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
+        <v>24</v>
+      </c>
+      <c r="O58" t="n">
+        <v>49</v>
+      </c>
+      <c r="P58" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>9</v>
+      </c>
+      <c r="R58" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S58" s="2" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="T58" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="U58" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="V58" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W58" s="2" t="n">
+        <v>-0.01636958628892898</v>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.150x154; O/U:Over@0.120x129</t>
+        </is>
+      </c>
+      <c r="Z58" t="n">
+        <v>-56.5</v>
+      </c>
+      <c r="AA58" t="n">
+        <v>-28.29</v>
+      </c>
+      <c r="AB58" t="inlineStr"/>
+      <c r="AC58" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD58" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>14:33:47</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>14</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>3-11</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="n">
+        <v>0.0465</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>0.0232</v>
+      </c>
+      <c r="J59" t="n">
+        <v>11900</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N59" t="n">
+        <v>27</v>
+      </c>
+      <c r="O59" t="n">
+        <v>54</v>
+      </c>
+      <c r="P59" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>9</v>
+      </c>
+      <c r="R59" t="n">
+        <v>-3</v>
+      </c>
+      <c r="S59" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="T59" s="2" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="U59" s="2" t="n"/>
+      <c r="V59" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W59" s="2" t="n">
+        <v>-0.03676212713122368</v>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.150x154; O/U:Over@0.120x129</t>
+        </is>
+      </c>
+      <c r="Z59" t="n">
+        <v>-56.5</v>
+      </c>
+      <c r="AA59" t="n">
+        <v>-12.91</v>
+      </c>
+      <c r="AB59" t="inlineStr"/>
+      <c r="AC59" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD59" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6368,7 +6905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7371,6 +7908,57 @@
         <v>0</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>14:30:56</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>11</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>O/U</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>129.0833333333333</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>0.2640755772590637</v>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>0.1140755772590637</v>
+      </c>
+      <c r="M20" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 14:39:37 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD59"/>
+  <dimension ref="A1:AD62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6894,6 +6894,329 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>14:36:05</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>15</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>3-12</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>0.0237</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>0.0118</v>
+      </c>
+      <c r="J60" t="n">
+        <v>9500</v>
+      </c>
+      <c r="K60" t="n">
+        <v>7400</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N60" t="n">
+        <v>29</v>
+      </c>
+      <c r="O60" t="n">
+        <v>59</v>
+      </c>
+      <c r="P60" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>10</v>
+      </c>
+      <c r="R60" t="n">
+        <v>-4</v>
+      </c>
+      <c r="S60" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="T60" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="U60" s="2" t="n"/>
+      <c r="V60" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W60" s="2" t="n">
+        <v>-0.02815915174782276</v>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.150x154; O/U:Over@0.120x129</t>
+        </is>
+      </c>
+      <c r="Z60" t="n">
+        <v>-56.5</v>
+      </c>
+      <c r="AA60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB60" t="inlineStr"/>
+      <c r="AC60" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD60" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>14:38:01</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>2</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>16</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>4-12</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="n">
+        <v>0.0108</v>
+      </c>
+      <c r="I61" s="2" t="n">
+        <v>0.0054</v>
+      </c>
+      <c r="J61" t="n">
+        <v>9600</v>
+      </c>
+      <c r="K61" t="n">
+        <v>1800</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N61" t="n">
+        <v>31</v>
+      </c>
+      <c r="O61" t="n">
+        <v>62</v>
+      </c>
+      <c r="P61" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>10</v>
+      </c>
+      <c r="R61" t="n">
+        <v>-5</v>
+      </c>
+      <c r="S61" s="2" t="n">
+        <v>0.0055</v>
+      </c>
+      <c r="T61" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="U61" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="V61" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W61" s="2" t="n">
+        <v>-0.03437948962301016</v>
+      </c>
+      <c r="Y61" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132; MAP2:ECSTATIC@0.150x154; O/U:Over@0.120x129</t>
+        </is>
+      </c>
+      <c r="Z61" t="n">
+        <v>-56.5</v>
+      </c>
+      <c r="AA61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB61" t="inlineStr"/>
+      <c r="AC61" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD61" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>14:38:12</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>16</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>4-12</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>0.0108</v>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>0.0054</v>
+      </c>
+      <c r="J62" t="n">
+        <v>9600</v>
+      </c>
+      <c r="K62" t="n">
+        <v>1800</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N62" t="n">
+        <v>31</v>
+      </c>
+      <c r="O62" t="n">
+        <v>62</v>
+      </c>
+      <c r="P62" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>10</v>
+      </c>
+      <c r="R62" t="n">
+        <v>-5</v>
+      </c>
+      <c r="S62" s="2" t="n">
+        <v>0.0055</v>
+      </c>
+      <c r="T62" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="U62" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="V62" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W62" s="2" t="n">
+        <v>-0.03437948962301016</v>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z62" t="n">
+        <v>-103.26</v>
+      </c>
+      <c r="AA62" t="n">
+        <v>-38.27</v>
+      </c>
+      <c r="AB62" s="4" t="inlineStr">
+        <is>
+          <t>FORCE-EXIT MAP2 ECSTATIC P/L:$-27.53  FORCE-EXIT O/U Over P/L:$-19.23</t>
+        </is>
+      </c>
+      <c r="AC62" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD62" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6905,7 +7228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6917,7 +7240,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
@@ -7959,6 +8282,108 @@
         <v>0</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>14:38:12</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>16</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>MAP2</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>FORCE-EXIT</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>153.78</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>0.01075897924602032</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>0.009758979246020316</v>
+      </c>
+      <c r="M21" s="9" t="n">
+        <v>-27.52662</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>14:38:12</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>16</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>O/U</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>FORCE-EXIT</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Over</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>129.0833333333333</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>0.01075897924602032</v>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>0.009758979246020316</v>
+      </c>
+      <c r="M22" s="9" t="n">
+        <v>-19.23341666666667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
live update 14:44:47 UTC
</commit_message>
<xml_diff>
--- a/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
+++ b/data/live_logs/live_cs2-ecs-nem-2026-04-03_20260403_121753.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD62"/>
+  <dimension ref="A1:AD68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -469,7 +469,7 @@
     <col width="6" customWidth="1" min="16" max="16"/>
     <col width="6" customWidth="1" min="17" max="17"/>
     <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
@@ -7212,6 +7212,666 @@
         </is>
       </c>
       <c r="AD62" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>14:40:40</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>17</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>5-12</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="I63" s="2" t="n">
+        <v>0.008500000000000001</v>
+      </c>
+      <c r="J63" t="n">
+        <v>1900</v>
+      </c>
+      <c r="K63" t="n">
+        <v>4600</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N63" t="n">
+        <v>36</v>
+      </c>
+      <c r="O63" t="n">
+        <v>66</v>
+      </c>
+      <c r="P63" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>10</v>
+      </c>
+      <c r="R63" t="n">
+        <v>1</v>
+      </c>
+      <c r="S63" s="2" t="n">
+        <v>0.0355</v>
+      </c>
+      <c r="T63" s="2" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="U63" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="V63" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W63" s="2" t="n">
+        <v>-0.03648217215389013</v>
+      </c>
+      <c r="X63" s="2" t="n">
+        <v>-0.01596434430778024</v>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z63" t="n">
+        <v>-103.26</v>
+      </c>
+      <c r="AA63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB63" t="inlineStr"/>
+      <c r="AC63" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD63" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>14:42:05</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>17</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>6-12</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>0.008500000000000001</v>
+      </c>
+      <c r="J64" t="n">
+        <v>1900</v>
+      </c>
+      <c r="K64" t="n">
+        <v>4600</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N64" t="n">
+        <v>36</v>
+      </c>
+      <c r="O64" t="n">
+        <v>66</v>
+      </c>
+      <c r="P64" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>10</v>
+      </c>
+      <c r="R64" t="n">
+        <v>1</v>
+      </c>
+      <c r="S64" s="2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="T64" s="2" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="U64" s="2" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="V64" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W64" s="2" t="n">
+        <v>-0.03148217215389013</v>
+      </c>
+      <c r="X64" s="2" t="n">
+        <v>-0.01696434430778024</v>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z64" t="n">
+        <v>-103.26</v>
+      </c>
+      <c r="AA64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB64" t="inlineStr"/>
+      <c r="AC64" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD64" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>14:42:16</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>18</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>6-12</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="n">
+        <v>0.0287</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>0.0143</v>
+      </c>
+      <c r="J65" t="n">
+        <v>6200</v>
+      </c>
+      <c r="K65" t="n">
+        <v>9300</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N65" t="n">
+        <v>41</v>
+      </c>
+      <c r="O65" t="n">
+        <v>70</v>
+      </c>
+      <c r="P65" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>10</v>
+      </c>
+      <c r="R65" t="n">
+        <v>2</v>
+      </c>
+      <c r="S65" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="T65" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="U65" s="2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="V65" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W65" s="2" t="n">
+        <v>-0.02434214320033787</v>
+      </c>
+      <c r="X65" s="2" t="n">
+        <v>-0.05768428640067577</v>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z65" t="n">
+        <v>-103.26</v>
+      </c>
+      <c r="AA65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB65" t="inlineStr"/>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD65" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>14:43:20</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>19</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>7-12</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>0.0334</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>0.0167</v>
+      </c>
+      <c r="J66" t="n">
+        <v>8950</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N66" t="n">
+        <v>46</v>
+      </c>
+      <c r="O66" t="n">
+        <v>70</v>
+      </c>
+      <c r="P66" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>10</v>
+      </c>
+      <c r="R66" t="n">
+        <v>3</v>
+      </c>
+      <c r="S66" s="2" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="T66" s="2" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="U66" s="2" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="V66" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W66" s="2" t="n">
+        <v>-0.02568135076761244</v>
+      </c>
+      <c r="X66" s="2" t="n">
+        <v>-0.0433627015352249</v>
+      </c>
+      <c r="Y66" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z66" t="n">
+        <v>-103.26</v>
+      </c>
+      <c r="AA66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB66" t="inlineStr"/>
+      <c r="AC66" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD66" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>14:44:34</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>19</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>8-12</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="n">
+        <v>0.0334</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>0.0167</v>
+      </c>
+      <c r="J67" t="n">
+        <v>8950</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>pistol</t>
+        </is>
+      </c>
+      <c r="N67" t="n">
+        <v>46</v>
+      </c>
+      <c r="O67" t="n">
+        <v>70</v>
+      </c>
+      <c r="P67" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>10</v>
+      </c>
+      <c r="R67" t="n">
+        <v>3</v>
+      </c>
+      <c r="S67" s="2" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="T67" s="2" t="n">
+        <v>0.089</v>
+      </c>
+      <c r="U67" s="2" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="V67" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W67" s="2" t="n">
+        <v>-0.02568135076761244</v>
+      </c>
+      <c r="X67" s="2" t="n">
+        <v>0.01663729846477505</v>
+      </c>
+      <c r="Y67" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z67" t="n">
+        <v>-103.26</v>
+      </c>
+      <c r="AA67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB67" t="inlineStr"/>
+      <c r="AC67" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD67" t="inlineStr">
+        <is>
+          <t>Nemesis</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>14:44:46</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>20</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>8-12</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>0.0569</v>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>0.0285</v>
+      </c>
+      <c r="J68" t="n">
+        <v>11700</v>
+      </c>
+      <c r="K68" t="n">
+        <v>5400</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>eco</t>
+        </is>
+      </c>
+      <c r="N68" t="n">
+        <v>51</v>
+      </c>
+      <c r="O68" t="n">
+        <v>73</v>
+      </c>
+      <c r="P68" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>10</v>
+      </c>
+      <c r="R68" t="n">
+        <v>4</v>
+      </c>
+      <c r="S68" s="2" t="n">
+        <v>0.0605</v>
+      </c>
+      <c r="T68" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="U68" s="2" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="V68" t="n">
+        <v>10749.5716</v>
+      </c>
+      <c r="W68" s="2" t="n">
+        <v>-0.01747116626799103</v>
+      </c>
+      <c r="X68" s="2" t="n">
+        <v>0.01405766746401785</v>
+      </c>
+      <c r="Y68" t="inlineStr">
+        <is>
+          <t>MAP1:ECSTATIC@0.760x132</t>
+        </is>
+      </c>
+      <c r="Z68" t="n">
+        <v>-103.26</v>
+      </c>
+      <c r="AA68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB68" t="inlineStr"/>
+      <c r="AC68" t="inlineStr">
+        <is>
+          <t>ECSTATIC</t>
+        </is>
+      </c>
+      <c r="AD68" t="inlineStr">
         <is>
           <t>Nemesis</t>
         </is>

</xml_diff>